<commit_message>
Correction de l'erreur de Région (VPC/Subnet non trouvés)
</commit_message>
<xml_diff>
--- a/Feuille-excel/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille-excel/Feuille de calcul de la base de connaissance-1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anna\Documents\ODC\Feuille excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anna\Documents\ODC\Feuille-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F215CE7-4066-43DF-87F5-55088AECBA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB5198B-6633-4DA9-813F-13FA9B8A293A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1980,11 +1980,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="I9:I11"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="H6:H8"/>
     <mergeCell ref="I6:I8"/>
@@ -1998,6 +1993,11 @@
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="I9:I11"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
@@ -2064,6 +2064,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -2286,36 +2301,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2338,9 +2327,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Docs: Résolution conflit AWS CLI v1/v2 et corruption config
</commit_message>
<xml_diff>
--- a/Feuille-excel/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille-excel/Feuille de calcul de la base de connaissance-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anna\Documents\ODC\Feuille-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB5198B-6633-4DA9-813F-13FA9B8A293A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A87E1E-9B66-41B4-92AB-7FA53FE90977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="99">
   <si>
     <t>Commentaires</t>
   </si>
@@ -419,6 +419,36 @@
   </si>
   <si>
     <t>PB.5</t>
+  </si>
+  <si>
+    <t>Utilisation d'Auto Scaling dans AWS (Linux) Creation d'une instance EC2</t>
+  </si>
+  <si>
+    <t>Blocage total de la CLI AWS empêchant le lancement de l'instance</t>
+  </si>
+  <si>
+    <t>ascii' codec can't decode / Échec aws ec2 run-instances</t>
+  </si>
+  <si>
+    <t>1. Obsolescence : Conflit d'encodage avec l'ancienne version AWS CLI v1 (Python 2.7)
+2. Config : Mixage entre clés AWS et ID de Security Group dans le fichier credentials.</t>
+  </si>
+  <si>
+    <t>1. Upgrade : Installation forcée de la AWS CLI v2.
+2. Purge : Suppression et recréation des fichiers config et credentials.
+3. Validation : Utilisation du chemin absolu /usr/local/bin/aws pour garantir l'usage de la v2.</t>
+  </si>
+  <si>
+    <t>• AWS CLI v2 Installer (via curl et unzip)
+• Commande which aws (pour localiser l'exécutable)
+• Éditeur vi (pour nettoyer les fichiers cachés ~/.aws/)
+• Documentation AWS CLI (pour les variables d'environnement)</t>
+  </si>
+  <si>
+    <t>Probleme 6</t>
+  </si>
+  <si>
+    <t>L'erreur 'ascii' était trompeuse : elle masquait un conflit entre Python 2.7 (CLI v1) et les nouveaux formats de tokens AWS. La solution radicale (purge complète + installation de la v2 dans /usr/local/bin/) est la seule méthode fiable pour stabiliser l'environnement.</t>
   </si>
 </sst>
 </file>
@@ -682,7 +712,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -756,7 +786,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -766,6 +796,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1124,9 +1157,9 @@
     <col min="4" max="4" width="130.1796875" style="2" customWidth="1"/>
     <col min="5" max="5" width="148.54296875" style="2" customWidth="1"/>
     <col min="6" max="6" width="126.6328125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="114.6328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="227.26953125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="61.6328125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="96.26953125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="255.6328125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="83.6328125" style="2" customWidth="1"/>
     <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
@@ -1274,38 +1307,38 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C6" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="25" t="s">
+      <c r="H6" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="29" t="s">
+      <c r="I6" s="30" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="40" customHeight="1">
-      <c r="A7" s="31"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="32"/>
+      <c r="A7" s="32"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="33"/>
       <c r="D7" s="26"/>
       <c r="E7" s="26"/>
       <c r="F7" s="26"/>
@@ -1314,9 +1347,9 @@
       <c r="I7" s="27"/>
     </row>
     <row r="8" spans="1:9" ht="40" customHeight="1">
-      <c r="A8" s="31"/>
-      <c r="B8" s="34"/>
-      <c r="C8" s="32"/>
+      <c r="A8" s="32"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="33"/>
       <c r="D8" s="26"/>
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
@@ -1328,10 +1361,10 @@
       <c r="A9" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="33" t="s">
         <v>56</v>
       </c>
       <c r="D9" s="26" t="s">
@@ -1355,8 +1388,8 @@
     </row>
     <row r="10" spans="1:9" ht="22.5" customHeight="1">
       <c r="A10" s="28"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
       <c r="D10" s="26"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
@@ -1366,8 +1399,8 @@
     </row>
     <row r="11" spans="1:9" ht="22.5" customHeight="1">
       <c r="A11" s="28"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
       <c r="D11" s="26"/>
       <c r="E11" s="26"/>
       <c r="F11" s="26"/>
@@ -1462,8 +1495,32 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="22.5">
+    <row r="15" spans="1:9" ht="140">
       <c r="A15" s="4"/>
+      <c r="B15" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I15" s="24" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="22.5">
       <c r="A16" s="4"/>
@@ -1980,6 +2037,10 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="I9:I11"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="H6:H8"/>
     <mergeCell ref="I6:I8"/>
@@ -1994,13 +2055,9 @@
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="D6:D8"/>
     <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="I9:I11"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B6 B9 B12:B1048576" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
   </dataValidations>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>